<commit_message>
Update toolkit audience wording in downloads
</commit_message>
<xml_diff>
--- a/files/SME_Supplier_Quality_Readiness_Toolkit_Workbook.xlsx
+++ b/files/SME_Supplier_Quality_Readiness_Toolkit_Workbook.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R32ffccd925d24e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APQP Timeline" sheetId="2" r:id="R36216399d6fa4f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPAP Checklist" sheetId="3" r:id="R7c2269089bf549d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Scorecard" sheetId="4" r:id="R7d00d41d5fca47bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rc0459778504f4830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APQP Timeline" sheetId="2" r:id="Rf1aaff2e672b4969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PPAP Checklist" sheetId="3" r:id="R2c1ef94fe1a34c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Scorecard" sheetId="4" r:id="Rd0714cef99e64987"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -582,7 +582,7 @@
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>APQP Timeline for Manufacturers with Fewer Than 200 Employees</x:v>
+        <x:v>APQP Timeline for Small and Medium-Sized U.S. Manufacturers</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>

</xml_diff>